<commit_message>
Verify frozen D1 recovery journals and bounded minute input timing
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/validation/temporal_holdout_2026/outputs/source_data/Temporal_holdout_stage_B_source.xlsx
+++ b/Project 1 Data Quality Assessment/validation/temporal_holdout_2026/outputs/source_data/Temporal_holdout_stage_B_source.xlsx
@@ -2,17 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal scope" sheetId="1" r:id="Ra7a0a9d2cd4a442f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Information intervals" sheetId="2" r:id="R49e5a715a26b486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D2 synthetic" sheetId="3" r:id="R4e8e035a39d84c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D4 synthetic" sheetId="4" r:id="Re96d3a36ebe440ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D4 historical impact" sheetId="5" r:id="Rccf699d855454f52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D2 historical impact" sheetId="6" r:id="R071ddfd266464f72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D4 mapping replay" sheetId="7" r:id="Raaeb156ccbfb47e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D1 PLS replay" sheetId="8" r:id="R86b1a5dd570b4861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transform replay" sheetId="9" r:id="R3362a818481f49f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D5 context replay" sheetId="10" r:id="R503d80ed83f0403b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D3 replay" sheetId="11" r:id="Rcf22c2ec7c334c84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal scope" sheetId="1" r:id="Rd46a08b47ed0459c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Information intervals" sheetId="2" r:id="R481de05178944802"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D2 synthetic" sheetId="3" r:id="R0c3f5b7a187d429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D4 synthetic" sheetId="4" r:id="Ra652a229eeeb4669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D4 historical impact" sheetId="5" r:id="Rdcfaac86465e46c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D2 historical impact" sheetId="6" r:id="Rc2ffc54a712a4a4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D4 mapping replay" sheetId="7" r:id="R9a1628da591b47aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D1 PLS replay" sheetId="8" r:id="R9e334af8d02f4cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D1 recovery replay" sheetId="9" r:id="R39c288d3bb634c7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D1 recovery prefix" sheetId="10" r:id="Re735773afa334865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Minute alignment" sheetId="11" r:id="R5137e4a7cd944f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transform replay" sheetId="12" r:id="R45a48669b48f4069"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D5 context replay" sheetId="13" r:id="Rc40d50c79e5040c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D3 replay" sheetId="14" r:id="R0b93fdce4aa94238"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -406,37 +409,41 @@
     <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="62" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>month</x:v>
+        <x:v>sensor_id</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
-        <x:v>n_snapshots</x:v>
+        <x:v>cutoff_exclusive</x:v>
       </x:c>
       <x:c r="C1" s="5" t="str">
-        <x:v>posterior_max_abs_error</x:v>
+        <x:v>native_candidate_symmetric_difference</x:v>
       </x:c>
       <x:c r="D1" s="5" t="str">
-        <x:v>map_regime_mismatches</x:v>
+        <x:v>native_state_changed_hours</x:v>
       </x:c>
       <x:c r="E1" s="5" t="str">
-        <x:v>active_regime_mismatches</x:v>
+        <x:v>native_score_changed_hours</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
-        <x:v>state_mismatches</x:v>
+        <x:v>candidate_event_prefix_equal</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>candidate_output_changed_hours</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>2025-08</x:v>
-      </x:c>
-      <x:c r="B2" s="11" t="n">
-        <x:v>4464</x:v>
-      </x:c>
-      <x:c r="C2" s="13" t="n">
-        <x:v>5.551115123125784e-16</x:v>
+        <x:v>DO_1_1</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D2" s="11" t="n">
         <x:v>0</x:v>
@@ -444,19 +451,22 @@
       <x:c r="E2" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F2" s="11" t="n">
+      <x:c r="F2" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>2025-09</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="n">
-        <x:v>4320</x:v>
-      </x:c>
-      <x:c r="C3" s="13" t="n">
-        <x:v>7.771561172376097e-16</x:v>
+        <x:v>DO_1_1</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D3" s="11" t="n">
         <x:v>0</x:v>
@@ -464,19 +474,22 @@
       <x:c r="E3" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F3" s="11" t="n">
+      <x:c r="F3" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G3" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>2025-10</x:v>
-      </x:c>
-      <x:c r="B4" s="11" t="n">
-        <x:v>4464</x:v>
-      </x:c>
-      <x:c r="C4" s="13" t="n">
-        <x:v>2.05391259555654e-15</x:v>
+        <x:v>DO_1_1</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D4" s="11" t="n">
         <x:v>0</x:v>
@@ -484,19 +497,22 @@
       <x:c r="E4" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F4" s="11" t="n">
+      <x:c r="F4" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="6" t="str">
-        <x:v>2025-11</x:v>
-      </x:c>
-      <x:c r="B5" s="11" t="n">
-        <x:v>4320</x:v>
-      </x:c>
-      <x:c r="C5" s="13" t="n">
-        <x:v>1.2212453270876722e-15</x:v>
+        <x:v>DO_1_2</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="11" t="n">
         <x:v>0</x:v>
@@ -504,19 +520,22 @@
       <x:c r="E5" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F5" s="11" t="n">
+      <x:c r="F5" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="6" t="str">
-        <x:v>2025-12</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="n">
-        <x:v>4464</x:v>
-      </x:c>
-      <x:c r="C6" s="13" t="n">
-        <x:v>1.054711873393899e-15</x:v>
+        <x:v>DO_1_2</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="11" t="n">
         <x:v>0</x:v>
@@ -524,19 +543,22 @@
       <x:c r="E6" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F6" s="11" t="n">
+      <x:c r="F6" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="6" t="str">
-        <x:v>2026-01</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="n">
-        <x:v>4464</x:v>
-      </x:c>
-      <x:c r="C7" s="13" t="n">
-        <x:v>7.771561172376097e-16</x:v>
+        <x:v>DO_1_2</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="11" t="n">
         <x:v>0</x:v>
@@ -544,19 +566,22 @@
       <x:c r="E7" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F7" s="11" t="n">
+      <x:c r="F7" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="6" t="str">
-        <x:v>2026-02</x:v>
-      </x:c>
-      <x:c r="B8" s="11" t="n">
-        <x:v>4032</x:v>
-      </x:c>
-      <x:c r="C8" s="13" t="n">
-        <x:v>5.551115123125784e-16</x:v>
+        <x:v>DO_1_3</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="11" t="n">
         <x:v>0</x:v>
@@ -564,19 +589,22 @@
       <x:c r="E8" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F8" s="11" t="n">
+      <x:c r="F8" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="6" t="str">
-        <x:v>2026-03</x:v>
-      </x:c>
-      <x:c r="B9" s="11" t="n">
-        <x:v>4464</x:v>
-      </x:c>
-      <x:c r="C9" s="13" t="n">
-        <x:v>9.992007221626409e-16</x:v>
+        <x:v>DO_1_3</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="11" t="n">
         <x:v>0</x:v>
@@ -584,19 +612,22 @@
       <x:c r="E9" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F9" s="11" t="n">
+      <x:c r="F9" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="6" t="str">
-        <x:v>2026-04</x:v>
-      </x:c>
-      <x:c r="B10" s="11" t="n">
-        <x:v>1872</x:v>
-      </x:c>
-      <x:c r="C10" s="13" t="n">
-        <x:v>6.106226635438361e-16</x:v>
+        <x:v>DO_1_3</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="11" t="n">
         <x:v>0</x:v>
@@ -604,7 +635,769 @@
       <x:c r="E10" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F10" s="11" t="n">
+      <x:c r="F10" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>DO_1_4</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>DO_1_4</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>DO_1_4</x:v>
+      </x:c>
+      <x:c r="B13" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>DO_2_1</x:v>
+      </x:c>
+      <x:c r="B14" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>DO_2_1</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>DO_2_1</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>DO_2_2</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>DO_2_2</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>DO_2_2</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>DO_2_3</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C20" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G20" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="6" t="str">
+        <x:v>DO_2_3</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C21" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G21" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="6" t="str">
+        <x:v>DO_2_3</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C22" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G22" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="24" customHeight="1">
+      <x:c r="A23" s="6" t="str">
+        <x:v>DO_2_4</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G23" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24" s="6" t="str">
+        <x:v>DO_2_4</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C24" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D24" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G24" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="24" customHeight="1">
+      <x:c r="A25" s="6" t="str">
+        <x:v>DO_2_4</x:v>
+      </x:c>
+      <x:c r="B25" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C25" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D25" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F25" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G25" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="24" customHeight="1">
+      <x:c r="A26" s="6" t="str">
+        <x:v>ORP_1_1</x:v>
+      </x:c>
+      <x:c r="B26" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C26" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D26" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G26" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="24" customHeight="1">
+      <x:c r="A27" s="6" t="str">
+        <x:v>ORP_1_1</x:v>
+      </x:c>
+      <x:c r="B27" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D27" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G27" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28" s="6" t="str">
+        <x:v>ORP_1_1</x:v>
+      </x:c>
+      <x:c r="B28" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C28" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D28" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F28" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G28" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29" s="6" t="str">
+        <x:v>ORP_1_2</x:v>
+      </x:c>
+      <x:c r="B29" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C29" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G29" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="24" customHeight="1">
+      <x:c r="A30" s="6" t="str">
+        <x:v>ORP_1_2</x:v>
+      </x:c>
+      <x:c r="B30" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C30" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D30" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E30" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G30" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31" s="6" t="str">
+        <x:v>ORP_1_2</x:v>
+      </x:c>
+      <x:c r="B31" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C31" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D31" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G31" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="24" customHeight="1">
+      <x:c r="A32" s="6" t="str">
+        <x:v>ORP_1_3</x:v>
+      </x:c>
+      <x:c r="B32" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C32" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D32" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G32" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="24" customHeight="1">
+      <x:c r="A33" s="6" t="str">
+        <x:v>ORP_1_3</x:v>
+      </x:c>
+      <x:c r="B33" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C33" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D33" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F33" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G33" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="24" customHeight="1">
+      <x:c r="A34" s="6" t="str">
+        <x:v>ORP_1_3</x:v>
+      </x:c>
+      <x:c r="B34" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C34" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D34" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G34" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="24" customHeight="1">
+      <x:c r="A35" s="6" t="str">
+        <x:v>ORP_2_1</x:v>
+      </x:c>
+      <x:c r="B35" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C35" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D35" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G35" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="24" customHeight="1">
+      <x:c r="A36" s="6" t="str">
+        <x:v>ORP_2_1</x:v>
+      </x:c>
+      <x:c r="B36" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C36" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D36" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F36" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G36" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="24" customHeight="1">
+      <x:c r="A37" s="6" t="str">
+        <x:v>ORP_2_1</x:v>
+      </x:c>
+      <x:c r="B37" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C37" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D37" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E37" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F37" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G37" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="24" customHeight="1">
+      <x:c r="A38" s="6" t="str">
+        <x:v>ORP_2_2</x:v>
+      </x:c>
+      <x:c r="B38" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C38" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D38" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E38" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F38" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G38" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="6" t="str">
+        <x:v>ORP_2_2</x:v>
+      </x:c>
+      <x:c r="B39" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C39" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F39" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G39" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="24" customHeight="1">
+      <x:c r="A40" s="6" t="str">
+        <x:v>ORP_2_2</x:v>
+      </x:c>
+      <x:c r="B40" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C40" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F40" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G40" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="24" customHeight="1">
+      <x:c r="A41" s="6" t="str">
+        <x:v>ORP_2_3</x:v>
+      </x:c>
+      <x:c r="B41" s="7" t="n">
+        <x:v>46054</x:v>
+      </x:c>
+      <x:c r="C41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F41" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G41" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="24" customHeight="1">
+      <x:c r="A42" s="6" t="str">
+        <x:v>ORP_2_3</x:v>
+      </x:c>
+      <x:c r="B42" s="7" t="n">
+        <x:v>46082</x:v>
+      </x:c>
+      <x:c r="C42" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E42" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F42" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G42" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="24" customHeight="1">
+      <x:c r="A43" s="6" t="str">
+        <x:v>ORP_2_3</x:v>
+      </x:c>
+      <x:c r="B43" s="7" t="n">
+        <x:v>46113</x:v>
+      </x:c>
+      <x:c r="C43" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D43" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E43" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F43" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G43" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -614,6 +1407,1677 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="62" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>sensor_id</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>n_minutes</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>n_released_minutes</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>native_vs_archive_max_abs</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>native_vs_archive_NA_differences</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>native_vs_archive_flag_differences</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>archived_diagnostic_flag_replay_differences</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>candidate_vs_native_changed_minutes</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
+        <x:v>candidate_short_fill_count</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>range_ineligible_count</x:v>
+      </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>chunk_max_abs</x:v>
+      </x:c>
+      <x:c r="L1" s="5" t="str">
+        <x:v>chunk_NA_differences</x:v>
+      </x:c>
+      <x:c r="M1" s="5" t="str">
+        <x:v>chunk_flag_differences</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>DO_1_1</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="n">
+        <x:v>20377</x:v>
+      </x:c>
+      <x:c r="G2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I2" s="11" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="J2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>DO_1_2</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" s="11" t="n">
+        <x:v>21913</x:v>
+      </x:c>
+      <x:c r="G3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I3" s="11" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="J3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>DO_1_3</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="n">
+        <x:v>15302</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" s="11" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="J4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>DO_1_4</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="n">
+        <x:v>54890</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="11" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>DO_2_1</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="n">
+        <x:v>27099</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="11" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>DO_2_2</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="n">
+        <x:v>24660</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="11" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>DO_2_3</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="n">
+        <x:v>14814</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>DO_2_4</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="n">
+        <x:v>47184</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="11" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>ORP_1_1</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="n">
+        <x:v>19640</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>ORP_1_2</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="n">
+        <x:v>16770</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="11" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="J11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>ORP_1_3</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="11" t="n">
+        <x:v>14636</x:v>
+      </x:c>
+      <x:c r="G12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="J12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>ORP_2_1</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="11" t="n">
+        <x:v>39651</x:v>
+      </x:c>
+      <x:c r="G13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>ORP_2_2</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="11" t="n">
+        <x:v>14678</x:v>
+      </x:c>
+      <x:c r="G14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="J14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>ORP_2_3</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="11" t="n">
+        <x:v>14637</x:v>
+      </x:c>
+      <x:c r="G15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>QR_1</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="11" t="n">
+        <x:v>14585</x:v>
+      </x:c>
+      <x:c r="G16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J16" s="11" t="n">
+        <x:v>11490</x:v>
+      </x:c>
+      <x:c r="K16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>QR_2</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="11" t="n">
+        <x:v>13906</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="J17" s="11" t="n">
+        <x:v>55859</x:v>
+      </x:c>
+      <x:c r="K17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>QIR_1</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="11" t="n">
+        <x:v>19772</x:v>
+      </x:c>
+      <x:c r="G18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="J18" s="11" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="K18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>QIR_2</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="n">
+        <x:v>368637</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="11" t="n">
+        <x:v>14632</x:v>
+      </x:c>
+      <x:c r="G19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="11" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="J19" s="11" t="n">
+        <x:v>939</x:v>
+      </x:c>
+      <x:c r="K19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="62" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>sensor_id</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>group</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>selected_order</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>fixed_extra_stl_passes</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>subhourly_period_min</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>n_minutes</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>decomposition_max_error</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>decomposition_na_mismatches</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
+        <x:v>prefix_max_error</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>whitening_max_error</x:v>
+      </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>whitening_chunk_max_error</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>DO_1_1</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>aerobic_do</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J2" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>DO_1_2</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>aerobic_do</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D3" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="6"/>
+      <x:c r="F3" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J3" s="13" t="n">
+        <x:v>6.661338147750939e-16</x:v>
+      </x:c>
+      <x:c r="K3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>DO_1_3</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>aerobic_do</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E4" s="6"/>
+      <x:c r="F4" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J4" s="13" t="n">
+        <x:v>8.881784197001252e-16</x:v>
+      </x:c>
+      <x:c r="K4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>DO_1_4</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>postanoxic_do</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="6"/>
+      <x:c r="F5" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>DO_2_1</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>aerobic_do</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="6"/>
+      <x:c r="F6" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>DO_2_2</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>aerobic_do</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E7" s="6"/>
+      <x:c r="F7" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>DO_2_3</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>aerobic_do</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="6"/>
+      <x:c r="F8" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="13" t="n">
+        <x:v>8.881784197001252e-16</x:v>
+      </x:c>
+      <x:c r="K8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>DO_2_4</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>postanoxic_do</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="6"/>
+      <x:c r="F9" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="13" t="n">
+        <x:v>4.440892098500626e-16</x:v>
+      </x:c>
+      <x:c r="K9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>ORP_1_1</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>anoxic_orp</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="6"/>
+      <x:c r="F10" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="13" t="n">
+        <x:v>4.440892098500626e-16</x:v>
+      </x:c>
+      <x:c r="K10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>ORP_1_2</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>anoxic_orp</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="6"/>
+      <x:c r="F11" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>ORP_1_3</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>anoxic_orp</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E12" s="6"/>
+      <x:c r="F12" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="13" t="n">
+        <x:v>8.881784197001252e-16</x:v>
+      </x:c>
+      <x:c r="K12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>ORP_2_1</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>anoxic_orp</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E13" s="6"/>
+      <x:c r="F13" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="13" t="n">
+        <x:v>4.440892098500626e-16</x:v>
+      </x:c>
+      <x:c r="K13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>ORP_2_2</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>anoxic_orp</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="6"/>
+      <x:c r="F14" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J14" s="13" t="n">
+        <x:v>4.440892098500626e-16</x:v>
+      </x:c>
+      <x:c r="K14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>ORP_2_3</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>anoxic_orp</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E15" s="6"/>
+      <x:c r="F15" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J15" s="13" t="n">
+        <x:v>8.881784197001252e-16</x:v>
+      </x:c>
+      <x:c r="K15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>QR_1</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>flow</x:v>
+      </x:c>
+      <x:c r="C16" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E16" s="6"/>
+      <x:c r="F16" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="13" t="n">
+        <x:v>8.881784197001252e-16</x:v>
+      </x:c>
+      <x:c r="K16" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>QR_2</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>flow</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E17" s="6"/>
+      <x:c r="F17" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K17" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>QIR_1</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>flow</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="6"/>
+      <x:c r="F18" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="13" t="n">
+        <x:v>4.440892098500626e-16</x:v>
+      </x:c>
+      <x:c r="K18" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>QIR_2</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="str">
+        <x:v>flow</x:v>
+      </x:c>
+      <x:c r="C19" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E19" s="6"/>
+      <x:c r="F19" s="11" t="n">
+        <x:v>368640</x:v>
+      </x:c>
+      <x:c r="G19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="13" t="n">
+        <x:v>4.440892098500626e-16</x:v>
+      </x:c>
+      <x:c r="K19" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="62" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>month</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>n_snapshots</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>posterior_max_abs_error</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>map_regime_mismatches</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>active_regime_mismatches</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>state_mismatches</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>2025-08</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="n">
+        <x:v>4464</x:v>
+      </x:c>
+      <x:c r="C2" s="13" t="n">
+        <x:v>5.551115123125784e-16</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>2025-09</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="n">
+        <x:v>4320</x:v>
+      </x:c>
+      <x:c r="C3" s="13" t="n">
+        <x:v>7.771561172376097e-16</x:v>
+      </x:c>
+      <x:c r="D3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>2025-10</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="n">
+        <x:v>4464</x:v>
+      </x:c>
+      <x:c r="C4" s="13" t="n">
+        <x:v>2.05391259555654e-15</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>2025-11</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="n">
+        <x:v>4320</x:v>
+      </x:c>
+      <x:c r="C5" s="13" t="n">
+        <x:v>1.2212453270876722e-15</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>2025-12</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="n">
+        <x:v>4464</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="n">
+        <x:v>1.054711873393899e-15</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>2026-01</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="n">
+        <x:v>4464</x:v>
+      </x:c>
+      <x:c r="C7" s="13" t="n">
+        <x:v>7.771561172376097e-16</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>2026-02</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="n">
+        <x:v>4032</x:v>
+      </x:c>
+      <x:c r="C8" s="13" t="n">
+        <x:v>5.551115123125784e-16</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>2026-03</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="n">
+        <x:v>4464</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="n">
+        <x:v>9.992007221626409e-16</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>2026-04</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="n">
+        <x:v>1872</x:v>
+      </x:c>
+      <x:c r="C10" s="13" t="n">
+        <x:v>6.106226635438361e-16</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -8440,6 +10904,15 @@
     <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="23" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="23" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="23" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="23" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="23" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="23" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="23" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="23" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="62" customHeight="1">
@@ -8447,52 +10920,81 @@
         <x:v>sensor_id</x:v>
       </x:c>
       <x:c r="B1" s="5" t="str">
-        <x:v>group</x:v>
+        <x:v>n_hours</x:v>
       </x:c>
       <x:c r="C1" s="5" t="str">
-        <x:v>selected_order</x:v>
+        <x:v>native_state_changed_hours</x:v>
       </x:c>
       <x:c r="D1" s="5" t="str">
-        <x:v>fixed_extra_stl_passes</x:v>
+        <x:v>native_state_max_abs_difference</x:v>
       </x:c>
       <x:c r="E1" s="5" t="str">
-        <x:v>subhourly_period_min</x:v>
+        <x:v>native_D1_max_abs_difference</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
-        <x:v>n_minutes</x:v>
+        <x:v>native_drift_max_abs_difference</x:v>
       </x:c>
       <x:c r="G1" s="5" t="str">
-        <x:v>decomposition_max_error</x:v>
+        <x:v>native_veto_changed_hours</x:v>
       </x:c>
       <x:c r="H1" s="5" t="str">
-        <x:v>decomposition_na_mismatches</x:v>
+        <x:v>native_NA_mismatches</x:v>
       </x:c>
       <x:c r="I1" s="5" t="str">
-        <x:v>prefix_max_error</x:v>
+        <x:v>native_transitions_equal</x:v>
       </x:c>
       <x:c r="J1" s="5" t="str">
-        <x:v>whitening_max_error</x:v>
+        <x:v>native_pelt_events_equal</x:v>
       </x:c>
       <x:c r="K1" s="5" t="str">
-        <x:v>whitening_chunk_max_error</x:v>
+        <x:v>native_event_count</x:v>
+      </x:c>
+      <x:c r="L1" s="5" t="str">
+        <x:v>scheduled_event_count</x:v>
+      </x:c>
+      <x:c r="M1" s="5" t="str">
+        <x:v>scheduled_score_changed_hours</x:v>
+      </x:c>
+      <x:c r="N1" s="5" t="str">
+        <x:v>scheduled_low_tail_flips</x:v>
+      </x:c>
+      <x:c r="O1" s="5" t="str">
+        <x:v>scheduled_state_changed_hours</x:v>
+      </x:c>
+      <x:c r="P1" s="5" t="str">
+        <x:v>checkpoint_output_changed_hours</x:v>
+      </x:c>
+      <x:c r="Q1" s="5" t="str">
+        <x:v>checkpoint_transitions_equal</x:v>
+      </x:c>
+      <x:c r="R1" s="5" t="str">
+        <x:v>incomplete_detector_hours</x:v>
+      </x:c>
+      <x:c r="S1" s="5" t="str">
+        <x:v>n_transitions</x:v>
+      </x:c>
+      <x:c r="T1" s="5" t="str">
+        <x:v>journal_sha256</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>DO_1_1</x:v>
       </x:c>
-      <x:c r="B2" s="6" t="str">
-        <x:v>aerobic_do</x:v>
+      <x:c r="B2" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C2" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D2" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E2" s="6"/>
+      <x:c r="E2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F2" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G2" s="11" t="n">
         <x:v>0</x:v>
@@ -8500,32 +11002,61 @@
       <x:c r="H2" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I2" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J2" s="13" t="n">
-        <x:v>0</x:v>
+      <x:c r="I2" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J2" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K2" s="11" t="n">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="L2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q2" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S2" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T2" s="6" t="str">
+        <x:v>1e993f5ded59052fd44829ba927bfe512c77ac16121a0ee2ebacb79db5f1ac75</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>DO_1_2</x:v>
       </x:c>
-      <x:c r="B3" s="6" t="str">
-        <x:v>aerobic_do</x:v>
+      <x:c r="B3" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C3" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D3" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E3" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F3" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G3" s="11" t="n">
         <x:v>0</x:v>
@@ -8533,65 +11064,123 @@
       <x:c r="H3" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I3" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J3" s="13" t="n">
-        <x:v>6.661338147750939e-16</x:v>
+      <x:c r="I3" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J3" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K3" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="L3" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="M3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q3" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R3" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S3" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="T3" s="6" t="str">
+        <x:v>8e94428d7c1e00c6377eb1f5e918a70ead147725c912415d4854dcbda28a4980</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>DO_1_3</x:v>
       </x:c>
-      <x:c r="B4" s="6" t="str">
-        <x:v>aerobic_do</x:v>
+      <x:c r="B4" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C4" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J4" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K4" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L4" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="M4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q4" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R4" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S4" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E4" s="6"/>
-      <x:c r="F4" s="11" t="n">
-        <x:v>368640</x:v>
-      </x:c>
-      <x:c r="G4" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H4" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I4" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J4" s="13" t="n">
-        <x:v>8.881784197001252e-16</x:v>
-      </x:c>
-      <x:c r="K4" s="11" t="n">
-        <x:v>0</x:v>
+      <x:c r="T4" s="6" t="str">
+        <x:v>b95c4e439e8ca87ef481e07e195cb7fc1f4166b3be99a5025d2ba7f93ddf6772</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>DO_1_4</x:v>
       </x:c>
-      <x:c r="B5" s="6" t="str">
-        <x:v>postanoxic_do</x:v>
+      <x:c r="B5" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C5" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E5" s="6"/>
+      <x:c r="E5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F5" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G5" s="11" t="n">
         <x:v>0</x:v>
@@ -8599,32 +11188,61 @@
       <x:c r="H5" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I5" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J5" s="13" t="n">
-        <x:v>0</x:v>
+      <x:c r="I5" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J5" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K5" s="11" t="n">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="L5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q5" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S5" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T5" s="6" t="str">
+        <x:v>a1fecf09f2d61487ca18cb496eed5e2f137d981a4e989a9fb3d2385016b9d413</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>DO_2_1</x:v>
       </x:c>
-      <x:c r="B6" s="6" t="str">
-        <x:v>aerobic_do</x:v>
+      <x:c r="B6" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C6" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F6" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="11" t="n">
         <x:v>0</x:v>
@@ -8632,32 +11250,61 @@
       <x:c r="H6" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I6" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J6" s="13" t="n">
-        <x:v>0</x:v>
+      <x:c r="I6" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J6" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K6" s="11" t="n">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="L6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q6" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S6" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T6" s="6" t="str">
+        <x:v>2e89d2e61a0ec6adf5c174556ba6853a662885adcdaeb381c6bf74af675594f4</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>DO_2_2</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="str">
-        <x:v>aerobic_do</x:v>
+      <x:c r="B7" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C7" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E7" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F7" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="11" t="n">
         <x:v>0</x:v>
@@ -8665,32 +11312,61 @@
       <x:c r="H7" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I7" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J7" s="13" t="n">
-        <x:v>0</x:v>
+      <x:c r="I7" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J7" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K7" s="11" t="n">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q7" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S7" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T7" s="6" t="str">
+        <x:v>8574c5ef1f6cd2c6f7aad9a1d38ca32d70ed5ad82873c3ebd82c1e95c8724b62</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>DO_2_3</x:v>
       </x:c>
-      <x:c r="B8" s="6" t="str">
-        <x:v>aerobic_do</x:v>
+      <x:c r="B8" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C8" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F8" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="11" t="n">
         <x:v>0</x:v>
@@ -8698,32 +11374,61 @@
       <x:c r="H8" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I8" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J8" s="13" t="n">
-        <x:v>8.881784197001252e-16</x:v>
+      <x:c r="I8" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J8" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K8" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="L8" s="11" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="M8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q8" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S8" s="11" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="T8" s="6" t="str">
+        <x:v>28655013907bb9a17cec8d73df271f30aa4b3d2fe9affa6b03f3c8291a43029c</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>DO_2_4</x:v>
       </x:c>
-      <x:c r="B9" s="6" t="str">
-        <x:v>postanoxic_do</x:v>
+      <x:c r="B9" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C9" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E9" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F9" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="11" t="n">
         <x:v>0</x:v>
@@ -8731,98 +11436,185 @@
       <x:c r="H9" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I9" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J9" s="13" t="n">
-        <x:v>4.440892098500626e-16</x:v>
+      <x:c r="I9" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J9" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K9" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="L9" s="11" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="M9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q9" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R9" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S9" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T9" s="6" t="str">
+        <x:v>18687f6d8e04028976ee38b0215350397735a048fdb8d9ebebb202c0ca8c464f</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>ORP_1_1</x:v>
       </x:c>
-      <x:c r="B10" s="6" t="str">
-        <x:v>anoxic_orp</x:v>
+      <x:c r="B10" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J10" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K10" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D10" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E10" s="6"/>
-      <x:c r="F10" s="11" t="n">
-        <x:v>368640</x:v>
-      </x:c>
-      <x:c r="G10" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H10" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I10" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J10" s="13" t="n">
-        <x:v>4.440892098500626e-16</x:v>
-      </x:c>
-      <x:c r="K10" s="11" t="n">
-        <x:v>0</x:v>
+      <x:c r="L10" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q10" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S10" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T10" s="6" t="str">
+        <x:v>fe12223fa9d9e58b71c62aea7c1ab75933b3ae0e56a3748d4c7cf81bfeff347d</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="6" t="str">
         <x:v>ORP_1_2</x:v>
       </x:c>
-      <x:c r="B11" s="6" t="str">
-        <x:v>anoxic_orp</x:v>
+      <x:c r="B11" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J11" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K11" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D11" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E11" s="6"/>
-      <x:c r="F11" s="11" t="n">
-        <x:v>368640</x:v>
-      </x:c>
-      <x:c r="G11" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H11" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I11" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J11" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K11" s="11" t="n">
-        <x:v>0</x:v>
+      <x:c r="L11" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q11" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R11" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S11" s="11" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="T11" s="6" t="str">
+        <x:v>a4fc66f1bb3d3fbec68094d51eda546cd2e21eb1d0c0407a13c3dcf0c04b6572</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>ORP_1_3</x:v>
       </x:c>
-      <x:c r="B12" s="6" t="str">
-        <x:v>anoxic_orp</x:v>
+      <x:c r="B12" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C12" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D12" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E12" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F12" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G12" s="11" t="n">
         <x:v>0</x:v>
@@ -8830,32 +11622,61 @@
       <x:c r="H12" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I12" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J12" s="13" t="n">
-        <x:v>8.881784197001252e-16</x:v>
+      <x:c r="I12" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J12" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K12" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="L12" s="11" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="M12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q12" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R12" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S12" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="T12" s="6" t="str">
+        <x:v>9ad08f55358f8b430539d5ba8b000911c7fbe83d8b9f155212d034c0943be526</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="6" t="str">
         <x:v>ORP_2_1</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="str">
-        <x:v>anoxic_orp</x:v>
+      <x:c r="B13" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C13" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D13" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E13" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F13" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="11" t="n">
         <x:v>0</x:v>
@@ -8863,32 +11684,61 @@
       <x:c r="H13" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I13" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J13" s="13" t="n">
-        <x:v>4.440892098500626e-16</x:v>
+      <x:c r="I13" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J13" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K13" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L13" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q13" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S13" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T13" s="6" t="str">
+        <x:v>bafe8ee36d2995f62d107982b45ce4f0a776a5a41ba0d46aa807094885fdcc84</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="6" t="str">
         <x:v>ORP_2_2</x:v>
       </x:c>
-      <x:c r="B14" s="6" t="str">
-        <x:v>anoxic_orp</x:v>
+      <x:c r="B14" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C14" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D14" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E14" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F14" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="11" t="n">
         <x:v>0</x:v>
@@ -8896,32 +11746,61 @@
       <x:c r="H14" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I14" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J14" s="13" t="n">
-        <x:v>4.440892098500626e-16</x:v>
+      <x:c r="I14" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J14" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K14" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L14" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q14" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R14" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S14" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="T14" s="6" t="str">
+        <x:v>3d74b631c7e9c059c87abf9f26e44947d81fee20615feee3b821df98e5eb75f6</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
         <x:v>ORP_2_3</x:v>
       </x:c>
-      <x:c r="B15" s="6" t="str">
-        <x:v>anoxic_orp</x:v>
+      <x:c r="B15" s="11" t="n">
+        <x:v>6138</x:v>
       </x:c>
       <x:c r="C15" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D15" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E15" s="6"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F15" s="11" t="n">
-        <x:v>368640</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="11" t="n">
         <x:v>0</x:v>
@@ -8929,146 +11808,41 @@
       <x:c r="H15" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I15" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J15" s="13" t="n">
-        <x:v>8.881784197001252e-16</x:v>
+      <x:c r="I15" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J15" s="10" t="b">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K15" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="6" t="str">
-        <x:v>QR_1</x:v>
-      </x:c>
-      <x:c r="B16" s="6" t="str">
-        <x:v>flow</x:v>
-      </x:c>
-      <x:c r="C16" s="11" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D16" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="11" t="n">
-        <x:v>368640</x:v>
-      </x:c>
-      <x:c r="G16" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H16" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I16" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J16" s="13" t="n">
-        <x:v>8.881784197001252e-16</x:v>
-      </x:c>
-      <x:c r="K16" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="6" t="str">
-        <x:v>QR_2</x:v>
-      </x:c>
-      <x:c r="B17" s="6" t="str">
-        <x:v>flow</x:v>
-      </x:c>
-      <x:c r="C17" s="11" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D17" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E17" s="6"/>
-      <x:c r="F17" s="11" t="n">
-        <x:v>368640</x:v>
-      </x:c>
-      <x:c r="G17" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H17" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I17" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J17" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K17" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="6" t="str">
-        <x:v>QIR_1</x:v>
-      </x:c>
-      <x:c r="B18" s="6" t="str">
-        <x:v>flow</x:v>
-      </x:c>
-      <x:c r="C18" s="11" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D18" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="6"/>
-      <x:c r="F18" s="11" t="n">
-        <x:v>368640</x:v>
-      </x:c>
-      <x:c r="G18" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H18" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I18" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J18" s="13" t="n">
-        <x:v>4.440892098500626e-16</x:v>
-      </x:c>
-      <x:c r="K18" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="6" t="str">
-        <x:v>QIR_2</x:v>
-      </x:c>
-      <x:c r="B19" s="6" t="str">
-        <x:v>flow</x:v>
-      </x:c>
-      <x:c r="C19" s="11" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D19" s="11" t="n">
+      <x:c r="L15" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E19" s="6"/>
-      <x:c r="F19" s="11" t="n">
-        <x:v>368640</x:v>
-      </x:c>
-      <x:c r="G19" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H19" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I19" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J19" s="13" t="n">
-        <x:v>4.440892098500626e-16</x:v>
-      </x:c>
-      <x:c r="K19" s="11" t="n">
-        <x:v>0</x:v>
+      <x:c r="M15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q15" s="10" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T15" s="6" t="str">
+        <x:v>90ecec0304d9e60b0b00f35c1e212035e4bb00232871f5ff2447cc477903b95e</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>